<commit_message>
Fix savings double count, align numbers, add charts and live demo link
- Season savings no longer add the batch value twice (EUR 239,310, not 354,810)
- Python rounding now matches the dashboard (35 waste batches), and the ROI
  chart uses the same monthly savings as the HACCP table
- HACCP_Impact_Simulation.csv is written by the pipeline, with the real
  deviation counts per parameter
- README rewritten with verified findings and charts; spec limits described
  as typical limits for 28-30 Brix aseptic paste
- charts/ folder with the 14 PNG charts, notebook links fixed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qy8CbYD8GTpf6MSCs4mucy
</commit_message>
<xml_diff>
--- a/tomato_qc_report.xlsx
+++ b/tomato_qc_report.xlsx
@@ -169,7 +169,7 @@
       <row>2</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7419975" cy="2524125"/>
+    <ext cx="7429500" cy="2533650"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -194,7 +194,7 @@
       <row>30</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2905125" cy="2809875"/>
+    <ext cx="2590800" cy="2819400"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -219,7 +219,7 @@
       <row>58</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4543425" cy="2809875"/>
+    <ext cx="4543425" cy="2819400"/>
     <pic>
       <nvPicPr>
         <cNvPr id="3" name="Image 3" descr="Picture"/>
@@ -244,7 +244,7 @@
       <row>86</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6267450" cy="3962400"/>
+    <ext cx="6267450" cy="3971925"/>
     <pic>
       <nvPicPr>
         <cNvPr id="4" name="Image 4" descr="Picture"/>
@@ -294,7 +294,7 @@
       <row>142</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7419975" cy="3095625"/>
+    <ext cx="7429500" cy="3105150"/>
     <pic>
       <nvPicPr>
         <cNvPr id="6" name="Image 6" descr="Picture"/>
@@ -344,7 +344,7 @@
       <row>198</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5114925" cy="3962400"/>
+    <ext cx="5114925" cy="3971925"/>
     <pic>
       <nvPicPr>
         <cNvPr id="8" name="Image 8" descr="Picture"/>
@@ -369,7 +369,7 @@
       <row>226</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7419975" cy="3952875"/>
+    <ext cx="7429500" cy="3971925"/>
     <pic>
       <nvPicPr>
         <cNvPr id="9" name="Image 9" descr="Picture"/>
@@ -394,7 +394,7 @@
       <row>254</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6267450" cy="3105150"/>
+    <ext cx="6276975" cy="3105150"/>
     <pic>
       <nvPicPr>
         <cNvPr id="10" name="Image 10" descr="Picture"/>
@@ -419,7 +419,7 @@
       <row>282</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7362825" cy="3371850"/>
+    <ext cx="7381875" cy="3390900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="11" name="Image 11" descr="Picture"/>
@@ -444,7 +444,7 @@
       <row>310</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8305800" cy="4210050"/>
+    <ext cx="8315325" cy="4210050"/>
     <pic>
       <nvPicPr>
         <cNvPr id="12" name="Image 12" descr="Picture"/>
@@ -469,7 +469,7 @@
       <row>338</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6267450" cy="3095625"/>
+    <ext cx="6276975" cy="3105150"/>
     <pic>
       <nvPicPr>
         <cNvPr id="13" name="Image 13" descr="Picture"/>
@@ -494,7 +494,7 @@
       <row>366</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5381625" cy="3952875"/>
+    <ext cx="5410200" cy="3971925"/>
     <pic>
       <nvPicPr>
         <cNvPr id="14" name="Image 14" descr="Picture"/>
@@ -48481,7 +48481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -48545,10 +48545,10 @@
         <v>589</v>
       </c>
       <c r="C5" t="n">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="D5" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6">
@@ -48577,10 +48577,10 @@
         <v>46</v>
       </c>
       <c r="C7" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D7" t="n">
-        <v>-12</v>
+        <v>-11</v>
       </c>
     </row>
     <row r="8">
@@ -48593,10 +48593,10 @@
         <v>93.61</v>
       </c>
       <c r="C8" t="n">
-        <v>95.28</v>
+        <v>95.14</v>
       </c>
       <c r="D8" t="n">
-        <v>1.67</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="9">
@@ -48625,10 +48625,10 @@
         <v>276000</v>
       </c>
       <c r="C10" t="n">
-        <v>204000</v>
+        <v>210000</v>
       </c>
       <c r="D10" t="n">
-        <v>-72000</v>
+        <v>-66000</v>
       </c>
     </row>
     <row r="11">
@@ -48641,10 +48641,10 @@
         <v>314250</v>
       </c>
       <c r="C11" t="n">
-        <v>228480</v>
+        <v>234480</v>
       </c>
       <c r="D11" t="n">
-        <v>-85770</v>
+        <v>-79770</v>
       </c>
     </row>
     <row r="12">
@@ -48657,10 +48657,10 @@
         <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>85770</v>
+        <v>79770</v>
       </c>
       <c r="D12" t="n">
-        <v>85770</v>
+        <v>79770</v>
       </c>
     </row>
     <row r="13">
@@ -48673,26 +48673,26 @@
         <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>257310</v>
+        <v>239310</v>
       </c>
       <c r="D13" t="n">
-        <v>257310</v>
+        <v>239310</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Annual revenue recovered (€)</t>
+          <t>Batch value saved, already inside annual savings (€)</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>126000</v>
+        <v>115500</v>
       </c>
       <c r="D14" t="n">
-        <v>126000</v>
+        <v>115500</v>
       </c>
     </row>
     <row r="17">
@@ -48930,42 +48930,49 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>HACCP = Hazard Analysis Critical Control Points (μηδενική ανοχή σε κρίσιμα CCPs)</t>
+          <t>HACCP = Hazard Analysis and Critical Control Points (zero tolerance at critical CCPs)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ISO 22000 = Διεθνές πρότυπο Food Safety Management System</t>
+          <t>ISO 22000 = international standard for food safety management systems</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Παραδοχή: -25% deviations &amp; waste μέσω CCP monitoring</t>
+          <t>Assumption: -25% deviations and waste through stronger CCP monitoring</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Παραδοχή: -15% operational cost μέσω physicochemical QC (Brix/pH/Acidity/Colour)</t>
+          <t>Assumption: -15% correction cost through physicochemical QC (Brix, pH, acidity, colour)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Annual projection = monthly savings × 3</t>
+          <t>Season projection = monthly savings x 3 production months</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Πηγή ποσοστών: εμπειρία D. Nomikos QC role</t>
+          <t>Batch value saved is part of the savings (the €6,000 waste cost includes the €3,500 batch), not extra</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Source of the reduction rates: my estimates from the D. Nomikos QC season</t>
         </is>
       </c>
     </row>

</xml_diff>